<commit_message>
Indexpruefung mit amtlichen Destatis-Werten hinterlegt
VPI Deutschland (2020=100): 04/2021 = 102,4; 04/2025 = 121,7; 07/2026 = 125,6.
Daraus zulaessige Miete zum fruehesten Anpassungstermin 14,86 EUR/qm gegenueber
der Forderung von 14,95 EUR/qm. Fuer das 1. OG betraegt die Indexveraenderung
seit 10/2023 nur 3,31 Prozent und liegt damit unter der Fuenfprozentschwelle.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Vergleich_Mietkonditionen_JN_DM.xlsx
+++ b/mietkonditionen/Vergleich_Mietkonditionen_JN_DM.xlsx
@@ -4504,18 +4504,22 @@
     <row r="122" hidden="1" outlineLevel="1">
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>VPI Übergabemonat 04/2021 (Destatis)</t>
-        </is>
-      </c>
-      <c r="C122" s="123" t="n"/>
+          <t>VPI 04/2021 – Basis 2./3. + 4. OG (Destatis)</t>
+        </is>
+      </c>
+      <c r="C122" s="123" t="n">
+        <v>102.4</v>
+      </c>
     </row>
     <row r="123" hidden="1" outlineLevel="1">
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>VPI Referenzmonat (Destatis)</t>
-        </is>
-      </c>
-      <c r="C123" s="123" t="n"/>
+          <t>VPI 04/2025 – frühester Anpassungstermin (Destatis)</t>
+        </is>
+      </c>
+      <c r="C123" s="123" t="n">
+        <v>121.7</v>
+      </c>
     </row>
     <row r="124" hidden="1" outlineLevel="1">
       <c r="B124" s="6" t="inlineStr">
@@ -4542,12 +4546,20 @@
     <row r="126" hidden="1" outlineLevel="1">
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>Basis 1. OG abweichend: 10/2023 (3. Nachtrag Ziff. 10)</t>
+          <t>Basis 1. OG: VPI 10/2023 = 117,8 → nur +3,31 %, unter der 5 %-Schwelle</t>
         </is>
       </c>
       <c r="C126" s="125" t="n"/>
     </row>
     <row r="127" hidden="1" outlineLevel="1">
+      <c r="B127" s="6" t="inlineStr">
+        <is>
+          <t>VPI 07/2026 – aktueller Stand (Destatis)</t>
+        </is>
+      </c>
+      <c r="C127" s="123" t="n">
+        <v>125.6</v>
+      </c>
       <c r="G127" s="52" t="n"/>
     </row>
     <row r="128" hidden="1" outlineLevel="1">

</xml_diff>

<commit_message>
Indexberechnung je Flaeche im Block 158-181 aufgebaut
Referenzwerte VPI (Destatis) als Eingabefelder, darunter eine Tabelle mit
allen acht indexrelevanten Positionen: die drei Mietflaechen, beide Keller
und die drei Stellplatzgruppen, jeweils mit eigenem Basismonat gemaess
3. Nachtrag Ziff. 10. Je Position wird die Indexveraenderung, die
Fuenfprozentschwelle und die zulaessige Miete berechnet.

Ergebnis zum Stichtag 04/2025: zulaessig 16.780,94 statt 14.910,75 EUR im
Monat. Die Forderung von 14,95 EUR/qm pauschal ergibt 16.513,77 EUR allein
fuer die Flaechen; davon sind 929,22 EUR monatlich nicht durch die
Indexklausel gedeckt, weil 1. OG und Keller 70 qm unter der Schwelle liegen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Vergleich_Mietkonditionen_JN_DM.xlsx
+++ b/mietkonditionen/Vergleich_Mietkonditionen_JN_DM.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -93,6 +93,14 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -144,7 +152,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -535,11 +543,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -765,18 +779,6 @@
     <xf numFmtId="164" fontId="2" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -854,6 +856,33 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="9" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="9" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -865,12 +894,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -889,31 +918,32 @@
     <xf numFmtId="168" fontId="2" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="170" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="9" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="9" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1320,8 +1350,8 @@
     <col width="37.85546875" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
     <col width="34.85546875" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
     <col width="12.85546875" customWidth="1" style="2" min="4" max="6"/>
-    <col width="11.42578125" customWidth="1" style="2" min="7" max="10"/>
-    <col width="11.42578125" customWidth="1" style="2" min="11" max="16384"/>
+    <col width="11.42578125" customWidth="1" style="2" min="7" max="11"/>
+    <col width="11.42578125" customWidth="1" style="2" min="12" max="16384"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1604,11 +1634,11 @@
           <t>qm/Bett</t>
         </is>
       </c>
-      <c r="C21" s="81">
+      <c r="C21" s="77">
         <f>+C20/C15</f>
         <v/>
       </c>
-      <c r="D21" s="81">
+      <c r="D21" s="77">
         <f>+D20/D15</f>
         <v/>
       </c>
@@ -1977,7 +2007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L163"/>
+  <dimension ref="A2:L217"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="3.85546875" customWidth="1" style="2" min="1" max="1"/>
@@ -1988,7 +2018,8 @@
     <col width="12.85546875" customWidth="1" style="2" min="8" max="8"/>
     <col width="11.42578125" customWidth="1" style="2" min="9" max="9"/>
     <col width="12.85546875" bestFit="1" customWidth="1" style="2" min="10" max="11"/>
-    <col width="11.42578125" customWidth="1" style="2" min="12" max="16384"/>
+    <col width="11.42578125" customWidth="1" style="2" min="12" max="12"/>
+    <col width="11.42578125" customWidth="1" style="2" min="13" max="16384"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -2008,22 +2039,22 @@
           <t>Standort:</t>
         </is>
       </c>
-      <c r="C4" s="110" t="inlineStr">
+      <c r="C4" s="115" t="inlineStr">
         <is>
           <t>Würselen (Target)</t>
         </is>
       </c>
-      <c r="D4" s="111" t="n"/>
-      <c r="E4" s="111" t="n"/>
-      <c r="F4" s="112" t="n"/>
-      <c r="G4" s="113" t="inlineStr">
+      <c r="D4" s="116" t="n"/>
+      <c r="E4" s="116" t="n"/>
+      <c r="F4" s="117" t="n"/>
+      <c r="G4" s="119" t="inlineStr">
         <is>
           <t>Baesweiler (Bestand)</t>
         </is>
       </c>
-      <c r="H4" s="111" t="n"/>
-      <c r="I4" s="111" t="n"/>
-      <c r="J4" s="112" t="n"/>
+      <c r="H4" s="116" t="n"/>
+      <c r="I4" s="116" t="n"/>
+      <c r="J4" s="117" t="n"/>
     </row>
     <row r="5">
       <c r="G5" s="52" t="n"/>
@@ -2245,7 +2276,7 @@
       <c r="F15" s="72" t="n"/>
       <c r="G15" s="73" t="inlineStr">
         <is>
-          <t>XXX – 5 Jahre ab Mietbeginn</t>
+          <t>XXX – 5 Jahre ab Mietbeginn kündbar (unbefristet)</t>
         </is>
       </c>
       <c r="H15" s="26" t="n"/>
@@ -2333,7 +2364,7 @@
           <t>Aufschiebende Bedingung / Rücktrittsrecht</t>
         </is>
       </c>
-      <c r="C19" s="108" t="inlineStr">
+      <c r="C19" s="113" t="inlineStr">
         <is>
           <t>außerordentliche Kündigung bei &gt;3 Monate Verzug</t>
         </is>
@@ -2390,7 +2421,7 @@
       <c r="F21" s="26" t="n"/>
       <c r="G21" s="73" t="inlineStr">
         <is>
-          <t>keine; Miete 10 Jahre fest</t>
+          <t>für die ersten 10 Mietjahre keine. Danach offen</t>
         </is>
       </c>
       <c r="H21" s="26" t="n"/>
@@ -2452,22 +2483,22 @@
           <t>Mietsicherheit</t>
         </is>
       </c>
-      <c r="C24" s="108" t="inlineStr">
+      <c r="C24" s="113" t="inlineStr">
         <is>
           <t>Bankbürgschaft: 3 Bruttomonatsmieten.</t>
         </is>
       </c>
-      <c r="D24" s="109" t="n"/>
-      <c r="E24" s="109" t="n"/>
-      <c r="F24" s="109" t="n"/>
-      <c r="G24" s="114" t="inlineStr">
+      <c r="D24" s="114" t="n"/>
+      <c r="E24" s="114" t="n"/>
+      <c r="F24" s="114" t="n"/>
+      <c r="G24" s="118" t="inlineStr">
         <is>
           <t>Patronatserklärung: 1 Jahreskaltmiete.</t>
         </is>
       </c>
-      <c r="H24" s="109" t="n"/>
-      <c r="I24" s="109" t="n"/>
-      <c r="J24" s="109" t="n"/>
+      <c r="H24" s="114" t="n"/>
+      <c r="I24" s="114" t="n"/>
+      <c r="J24" s="114" t="n"/>
       <c r="L24" s="47" t="n"/>
     </row>
     <row r="25">
@@ -2600,13 +2631,13 @@
           <t>Miete/m² (Neubau) - kein BKZ</t>
         </is>
       </c>
-      <c r="C32" s="115" t="n">
+      <c r="C32" s="120" t="n">
         <v>20</v>
       </c>
       <c r="D32" s="26" t="n"/>
       <c r="E32" s="26" t="n"/>
       <c r="F32" s="26" t="n"/>
-      <c r="G32" s="116" t="n">
+      <c r="G32" s="121" t="n">
         <v>20</v>
       </c>
       <c r="H32" s="26" t="n"/>
@@ -2619,13 +2650,13 @@
           <t>Miete/m² inkl. BKZ</t>
         </is>
       </c>
-      <c r="C33" s="115" t="n">
+      <c r="C33" s="120" t="n">
         <v>20</v>
       </c>
       <c r="D33" s="26" t="n"/>
       <c r="E33" s="26" t="n"/>
       <c r="F33" s="26" t="n"/>
-      <c r="G33" s="116" t="n">
+      <c r="G33" s="121" t="n">
         <v>20</v>
       </c>
       <c r="H33" s="26" t="n"/>
@@ -2638,13 +2669,13 @@
           <t>Nebenkosten/m²</t>
         </is>
       </c>
-      <c r="C34" s="115" t="n">
+      <c r="C34" s="120" t="n">
         <v>3</v>
       </c>
       <c r="D34" s="26" t="n"/>
       <c r="E34" s="26" t="n"/>
       <c r="F34" s="26" t="n"/>
-      <c r="G34" s="116" t="n">
+      <c r="G34" s="121" t="n">
         <v>3</v>
       </c>
       <c r="H34" s="26" t="n"/>
@@ -2657,24 +2688,24 @@
           <t>Fläche pro Bett</t>
         </is>
       </c>
-      <c r="C35" s="117" t="inlineStr">
+      <c r="C35" s="122" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="D35" s="118" t="inlineStr">
+      <c r="D35" s="123" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
       </c>
       <c r="E35" s="26" t="n"/>
       <c r="F35" s="26" t="n"/>
-      <c r="G35" s="119" t="inlineStr">
+      <c r="G35" s="124" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="H35" s="118" t="inlineStr">
+      <c r="H35" s="123" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
@@ -2688,13 +2719,13 @@
           <t>Miete pro Bett pro Monat (exkl. Baukostenzuschuss)</t>
         </is>
       </c>
-      <c r="C36" s="117" t="n">
+      <c r="C36" s="122" t="n">
         <v>1000</v>
       </c>
       <c r="D36" s="26" t="n"/>
       <c r="E36" s="26" t="n"/>
       <c r="F36" s="26" t="n"/>
-      <c r="G36" s="119" t="n">
+      <c r="G36" s="124" t="n">
         <v>1000</v>
       </c>
       <c r="H36" s="26" t="n"/>
@@ -2707,14 +2738,14 @@
           <t>Miete pro Bett pro Monat (inkl. BKZ über 10 Jahre)</t>
         </is>
       </c>
-      <c r="C37" s="117">
+      <c r="C37" s="122">
         <f>+C36</f>
         <v/>
       </c>
       <c r="D37" s="26" t="n"/>
       <c r="E37" s="26" t="n"/>
       <c r="F37" s="26" t="n"/>
-      <c r="G37" s="119">
+      <c r="G37" s="124">
         <f>+G36</f>
         <v/>
       </c>
@@ -2728,16 +2759,16 @@
           <t>Baukostenzuschuss pro Bett</t>
         </is>
       </c>
-      <c r="C38" s="117" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="118" t="n"/>
+      <c r="C38" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="123" t="n"/>
       <c r="E38" s="26" t="n"/>
       <c r="F38" s="26" t="n"/>
-      <c r="G38" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="118" t="n"/>
+      <c r="G38" s="124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="123" t="n"/>
       <c r="I38" s="26" t="n"/>
       <c r="J38" s="26" t="n"/>
     </row>
@@ -2747,13 +2778,13 @@
           <t>Capex pro Bett (Möbel, Ausstattung, etc.)</t>
         </is>
       </c>
-      <c r="C39" s="117" t="n">
+      <c r="C39" s="122" t="n">
         <v>30000</v>
       </c>
       <c r="D39" s="26" t="n"/>
       <c r="E39" s="26" t="n"/>
       <c r="F39" s="26" t="n"/>
-      <c r="G39" s="119" t="n">
+      <c r="G39" s="124" t="n">
         <v>30000</v>
       </c>
       <c r="H39" s="26" t="n"/>
@@ -2807,13 +2838,13 @@
           <t>Miete/m² (Bestand) - kein BKZ</t>
         </is>
       </c>
-      <c r="C43" s="115" t="n">
+      <c r="C43" s="120" t="n">
         <v>20</v>
       </c>
       <c r="D43" s="26" t="n"/>
       <c r="E43" s="26" t="n"/>
       <c r="F43" s="26" t="n"/>
-      <c r="G43" s="116" t="n">
+      <c r="G43" s="121" t="n">
         <v>20</v>
       </c>
       <c r="H43" s="26" t="n"/>
@@ -2826,13 +2857,13 @@
           <t>Miete/m² (Bestand) inkl. BKZ</t>
         </is>
       </c>
-      <c r="C44" s="115" t="n">
+      <c r="C44" s="120" t="n">
         <v>25</v>
       </c>
       <c r="D44" s="26" t="n"/>
       <c r="E44" s="26" t="n"/>
       <c r="F44" s="26" t="n"/>
-      <c r="G44" s="116" t="n">
+      <c r="G44" s="121" t="n">
         <v>25</v>
       </c>
       <c r="H44" s="26" t="n"/>
@@ -2845,13 +2876,13 @@
           <t>Nebenkosten/m²</t>
         </is>
       </c>
-      <c r="C45" s="115" t="n">
+      <c r="C45" s="120" t="n">
         <v>3</v>
       </c>
       <c r="D45" s="26" t="n"/>
       <c r="E45" s="26" t="n"/>
       <c r="F45" s="26" t="n"/>
-      <c r="G45" s="116" t="n">
+      <c r="G45" s="121" t="n">
         <v>3</v>
       </c>
       <c r="H45" s="26" t="n"/>
@@ -2864,24 +2895,24 @@
           <t>Fläche pro Bett</t>
         </is>
       </c>
-      <c r="C46" s="117" t="inlineStr">
+      <c r="C46" s="122" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="D46" s="118" t="inlineStr">
+      <c r="D46" s="123" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
       </c>
       <c r="E46" s="26" t="n"/>
       <c r="F46" s="26" t="n"/>
-      <c r="G46" s="119" t="inlineStr">
+      <c r="G46" s="124" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="H46" s="118" t="inlineStr">
+      <c r="H46" s="123" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
@@ -2895,13 +2926,13 @@
           <t>Miete pro Bett pro Monat (exkl. Baukostenzuschuss)</t>
         </is>
       </c>
-      <c r="C47" s="117" t="n">
+      <c r="C47" s="122" t="n">
         <v>1000</v>
       </c>
       <c r="D47" s="26" t="n"/>
       <c r="E47" s="26" t="n"/>
       <c r="F47" s="26" t="n"/>
-      <c r="G47" s="119" t="n">
+      <c r="G47" s="124" t="n">
         <v>1000</v>
       </c>
       <c r="H47" s="26" t="n"/>
@@ -2914,13 +2945,13 @@
           <t>Miete pro Bett pro Monat (inkl. BKZ über 10 Jahre)</t>
         </is>
       </c>
-      <c r="C48" s="117" t="n">
+      <c r="C48" s="122" t="n">
         <v>1250</v>
       </c>
       <c r="D48" s="26" t="n"/>
       <c r="E48" s="26" t="n"/>
       <c r="F48" s="26" t="n"/>
-      <c r="G48" s="119" t="n">
+      <c r="G48" s="124" t="n">
         <v>1250</v>
       </c>
       <c r="H48" s="26" t="n"/>
@@ -2933,20 +2964,20 @@
           <t>Baukostenzuschuss pro Bett</t>
         </is>
       </c>
-      <c r="C49" s="117" t="n">
+      <c r="C49" s="122" t="n">
         <v>40000</v>
       </c>
-      <c r="D49" s="118" t="inlineStr">
+      <c r="D49" s="123" t="inlineStr">
         <is>
           <t>(d.h. 6er WG: 180.000 €, 12er WG: 360.000 €)</t>
         </is>
       </c>
       <c r="E49" s="26" t="n"/>
       <c r="F49" s="26" t="n"/>
-      <c r="G49" s="119" t="n">
+      <c r="G49" s="124" t="n">
         <v>40000</v>
       </c>
-      <c r="H49" s="118" t="inlineStr">
+      <c r="H49" s="123" t="inlineStr">
         <is>
           <t>(d.h. 6er WG: 180.000 €, 12er WG: 360.000 €)</t>
         </is>
@@ -2960,13 +2991,13 @@
           <t>Capex pro Bett (Möbel, Ausstattung, etc.)</t>
         </is>
       </c>
-      <c r="C50" s="117" t="n">
+      <c r="C50" s="122" t="n">
         <v>30000</v>
       </c>
       <c r="D50" s="26" t="n"/>
       <c r="E50" s="26" t="n"/>
       <c r="F50" s="26" t="n"/>
-      <c r="G50" s="119" t="n">
+      <c r="G50" s="124" t="n">
         <v>30000</v>
       </c>
       <c r="H50" s="26" t="n"/>
@@ -3335,7 +3366,7 @@
           <t>Keller</t>
         </is>
       </c>
-      <c r="C66" s="120" t="n">
+      <c r="C66" s="125" t="n">
         <v>18.65</v>
       </c>
       <c r="D66" s="33" t="n">
@@ -3461,10 +3492,10 @@
       <c r="D72" s="10" t="n"/>
       <c r="E72" s="10" t="n"/>
       <c r="F72" s="10" t="n"/>
-      <c r="G72" s="84" t="n"/>
-      <c r="H72" s="85" t="n"/>
-      <c r="I72" s="85" t="n"/>
-      <c r="J72" s="85" t="n"/>
+      <c r="G72" s="80" t="n"/>
+      <c r="H72" s="81" t="n"/>
+      <c r="I72" s="81" t="n"/>
+      <c r="J72" s="81" t="n"/>
     </row>
     <row r="73">
       <c r="B73" s="6" t="inlineStr">
@@ -3480,10 +3511,10 @@
       <c r="D73" s="26" t="n"/>
       <c r="E73" s="26" t="n"/>
       <c r="F73" s="26" t="n"/>
-      <c r="G73" s="86" t="n"/>
-      <c r="H73" s="87" t="n"/>
-      <c r="I73" s="87" t="n"/>
-      <c r="J73" s="87" t="n"/>
+      <c r="G73" s="82" t="n"/>
+      <c r="H73" s="83" t="n"/>
+      <c r="I73" s="83" t="n"/>
+      <c r="J73" s="83" t="n"/>
     </row>
     <row r="74">
       <c r="B74" s="6" t="inlineStr">
@@ -3499,10 +3530,10 @@
       <c r="D74" s="26" t="n"/>
       <c r="E74" s="26" t="n"/>
       <c r="F74" s="26" t="n"/>
-      <c r="G74" s="86" t="n"/>
-      <c r="H74" s="87" t="n"/>
-      <c r="I74" s="87" t="n"/>
-      <c r="J74" s="87" t="n"/>
+      <c r="G74" s="82" t="n"/>
+      <c r="H74" s="83" t="n"/>
+      <c r="I74" s="83" t="n"/>
+      <c r="J74" s="83" t="n"/>
     </row>
     <row r="75">
       <c r="B75" s="6" t="inlineStr">
@@ -3518,10 +3549,10 @@
       <c r="D75" s="26" t="n"/>
       <c r="E75" s="26" t="n"/>
       <c r="F75" s="26" t="n"/>
-      <c r="G75" s="86" t="n"/>
-      <c r="H75" s="87" t="n"/>
-      <c r="I75" s="87" t="n"/>
-      <c r="J75" s="87" t="n"/>
+      <c r="G75" s="82" t="n"/>
+      <c r="H75" s="83" t="n"/>
+      <c r="I75" s="83" t="n"/>
+      <c r="J75" s="83" t="n"/>
       <c r="L75" s="47" t="n"/>
     </row>
     <row r="76">
@@ -3536,10 +3567,10 @@
       <c r="D76" s="26" t="n"/>
       <c r="E76" s="26" t="n"/>
       <c r="F76" s="26" t="n"/>
-      <c r="G76" s="88" t="n"/>
-      <c r="H76" s="87" t="n"/>
-      <c r="I76" s="87" t="n"/>
-      <c r="J76" s="87" t="n"/>
+      <c r="G76" s="84" t="n"/>
+      <c r="H76" s="83" t="n"/>
+      <c r="I76" s="83" t="n"/>
+      <c r="J76" s="83" t="n"/>
     </row>
     <row r="77">
       <c r="B77" s="6" t="inlineStr">
@@ -3555,16 +3586,16 @@
       <c r="D77" s="26" t="n"/>
       <c r="E77" s="26" t="n"/>
       <c r="F77" s="26" t="n"/>
-      <c r="G77" s="89" t="n"/>
-      <c r="H77" s="87" t="n"/>
-      <c r="I77" s="87" t="n"/>
-      <c r="J77" s="87" t="n"/>
+      <c r="G77" s="85" t="n"/>
+      <c r="H77" s="83" t="n"/>
+      <c r="I77" s="83" t="n"/>
+      <c r="J77" s="83" t="n"/>
     </row>
     <row r="78">
-      <c r="G78" s="90" t="n"/>
-      <c r="H78" s="91" t="n"/>
-      <c r="I78" s="91" t="n"/>
-      <c r="J78" s="91" t="n"/>
+      <c r="G78" s="86" t="n"/>
+      <c r="H78" s="87" t="n"/>
+      <c r="I78" s="87" t="n"/>
+      <c r="J78" s="87" t="n"/>
     </row>
     <row r="79">
       <c r="B79" s="11" t="inlineStr">
@@ -3592,10 +3623,10 @@
           <t>€ pro Jahr</t>
         </is>
       </c>
-      <c r="G79" s="92" t="n"/>
-      <c r="H79" s="93" t="n"/>
-      <c r="I79" s="93" t="n"/>
-      <c r="J79" s="93" t="n"/>
+      <c r="G79" s="88" t="n"/>
+      <c r="H79" s="89" t="n"/>
+      <c r="I79" s="89" t="n"/>
+      <c r="J79" s="89" t="n"/>
     </row>
     <row r="80">
       <c r="B80" s="2" t="inlineStr">
@@ -3617,10 +3648,10 @@
         <f>+E80*12</f>
         <v/>
       </c>
-      <c r="G80" s="94" t="n"/>
-      <c r="H80" s="95" t="n"/>
-      <c r="I80" s="96" t="n"/>
-      <c r="J80" s="96" t="n"/>
+      <c r="G80" s="90" t="n"/>
+      <c r="H80" s="91" t="n"/>
+      <c r="I80" s="92" t="n"/>
+      <c r="J80" s="92" t="n"/>
     </row>
     <row r="81">
       <c r="B81" s="6" t="inlineStr">
@@ -3643,10 +3674,10 @@
         <f>+E81*12</f>
         <v/>
       </c>
-      <c r="G81" s="97" t="n"/>
-      <c r="H81" s="98" t="n"/>
-      <c r="I81" s="96" t="n"/>
-      <c r="J81" s="96" t="n"/>
+      <c r="G81" s="93" t="n"/>
+      <c r="H81" s="94" t="n"/>
+      <c r="I81" s="92" t="n"/>
+      <c r="J81" s="92" t="n"/>
     </row>
     <row r="82">
       <c r="B82" s="6" t="inlineStr">
@@ -3668,10 +3699,10 @@
         <f>+E82*12</f>
         <v/>
       </c>
-      <c r="G82" s="99" t="n"/>
-      <c r="H82" s="98" t="n"/>
-      <c r="I82" s="96" t="n"/>
-      <c r="J82" s="96" t="n"/>
+      <c r="G82" s="95" t="n"/>
+      <c r="H82" s="94" t="n"/>
+      <c r="I82" s="92" t="n"/>
+      <c r="J82" s="92" t="n"/>
     </row>
     <row r="83">
       <c r="B83" s="6" t="inlineStr">
@@ -3693,10 +3724,10 @@
         <f>+E83*12</f>
         <v/>
       </c>
-      <c r="G83" s="97" t="n"/>
-      <c r="H83" s="98" t="n"/>
-      <c r="I83" s="96" t="n"/>
-      <c r="J83" s="96" t="n"/>
+      <c r="G83" s="93" t="n"/>
+      <c r="H83" s="94" t="n"/>
+      <c r="I83" s="92" t="n"/>
+      <c r="J83" s="92" t="n"/>
     </row>
     <row r="84">
       <c r="B84" s="6" t="inlineStr">
@@ -3718,10 +3749,10 @@
         <f>+E84*12</f>
         <v/>
       </c>
-      <c r="G84" s="97" t="n"/>
-      <c r="H84" s="98" t="n"/>
-      <c r="I84" s="96" t="n"/>
-      <c r="J84" s="96" t="n"/>
+      <c r="G84" s="93" t="n"/>
+      <c r="H84" s="94" t="n"/>
+      <c r="I84" s="92" t="n"/>
+      <c r="J84" s="92" t="n"/>
     </row>
     <row r="85">
       <c r="B85" s="72" t="inlineStr">
@@ -3743,10 +3774,10 @@
         <f>+E85*12</f>
         <v/>
       </c>
-      <c r="G85" s="99" t="n"/>
-      <c r="H85" s="98" t="n"/>
-      <c r="I85" s="96" t="n"/>
-      <c r="J85" s="96" t="n"/>
+      <c r="G85" s="95" t="n"/>
+      <c r="H85" s="94" t="n"/>
+      <c r="I85" s="92" t="n"/>
+      <c r="J85" s="92" t="n"/>
     </row>
     <row r="86" ht="8.25" customHeight="1">
       <c r="B86" s="14" t="n"/>
@@ -3754,10 +3785,10 @@
       <c r="D86" s="16" t="n"/>
       <c r="E86" s="17" t="n"/>
       <c r="F86" s="17" t="n"/>
-      <c r="G86" s="100" t="n"/>
-      <c r="H86" s="101" t="n"/>
-      <c r="I86" s="102" t="n"/>
-      <c r="J86" s="102" t="n"/>
+      <c r="G86" s="96" t="n"/>
+      <c r="H86" s="97" t="n"/>
+      <c r="I86" s="98" t="n"/>
+      <c r="J86" s="98" t="n"/>
     </row>
     <row r="87" customFormat="1" s="1">
       <c r="B87" s="1" t="inlineStr">
@@ -3775,10 +3806,10 @@
         <f>+SUM(F80:F86)</f>
         <v/>
       </c>
-      <c r="G87" s="103" t="n"/>
-      <c r="H87" s="104" t="n"/>
-      <c r="I87" s="105" t="n"/>
-      <c r="J87" s="105" t="n"/>
+      <c r="G87" s="99" t="n"/>
+      <c r="H87" s="100" t="n"/>
+      <c r="I87" s="101" t="n"/>
+      <c r="J87" s="101" t="n"/>
     </row>
     <row r="88" ht="6.75" customHeight="1" thickBot="1">
       <c r="B88" s="7" t="n"/>
@@ -3786,16 +3817,16 @@
       <c r="D88" s="7" t="n"/>
       <c r="E88" s="7" t="n"/>
       <c r="F88" s="7" t="n"/>
-      <c r="G88" s="106" t="n"/>
-      <c r="H88" s="107" t="n"/>
-      <c r="I88" s="107" t="n"/>
-      <c r="J88" s="107" t="n"/>
+      <c r="G88" s="102" t="n"/>
+      <c r="H88" s="103" t="n"/>
+      <c r="I88" s="103" t="n"/>
+      <c r="J88" s="103" t="n"/>
     </row>
     <row r="89">
-      <c r="G89" s="90" t="n"/>
-      <c r="H89" s="91" t="n"/>
-      <c r="I89" s="91" t="n"/>
-      <c r="J89" s="91" t="n"/>
+      <c r="G89" s="86" t="n"/>
+      <c r="H89" s="87" t="n"/>
+      <c r="I89" s="87" t="n"/>
+      <c r="J89" s="87" t="n"/>
     </row>
     <row r="90">
       <c r="B90" s="10" t="inlineStr">
@@ -3807,10 +3838,10 @@
       <c r="D90" s="10" t="n"/>
       <c r="E90" s="10" t="n"/>
       <c r="F90" s="10" t="n"/>
-      <c r="G90" s="84" t="n"/>
-      <c r="H90" s="85" t="n"/>
-      <c r="I90" s="85" t="n"/>
-      <c r="J90" s="85" t="n"/>
+      <c r="G90" s="80" t="n"/>
+      <c r="H90" s="81" t="n"/>
+      <c r="I90" s="81" t="n"/>
+      <c r="J90" s="81" t="n"/>
     </row>
     <row r="91">
       <c r="B91" s="6" t="inlineStr">
@@ -3826,10 +3857,10 @@
       <c r="D91" s="26" t="n"/>
       <c r="E91" s="26" t="n"/>
       <c r="F91" s="26" t="n"/>
-      <c r="G91" s="86" t="n"/>
-      <c r="H91" s="87" t="n"/>
-      <c r="I91" s="87" t="n"/>
-      <c r="J91" s="87" t="n"/>
+      <c r="G91" s="82" t="n"/>
+      <c r="H91" s="83" t="n"/>
+      <c r="I91" s="83" t="n"/>
+      <c r="J91" s="83" t="n"/>
     </row>
     <row r="92">
       <c r="B92" s="6" t="inlineStr">
@@ -3845,10 +3876,10 @@
       <c r="D92" s="26" t="n"/>
       <c r="E92" s="26" t="n"/>
       <c r="F92" s="26" t="n"/>
-      <c r="G92" s="86" t="n"/>
-      <c r="H92" s="87" t="n"/>
-      <c r="I92" s="87" t="n"/>
-      <c r="J92" s="87" t="n"/>
+      <c r="G92" s="82" t="n"/>
+      <c r="H92" s="83" t="n"/>
+      <c r="I92" s="83" t="n"/>
+      <c r="J92" s="83" t="n"/>
       <c r="L92" s="47" t="n"/>
     </row>
     <row r="93">
@@ -3863,10 +3894,10 @@
       <c r="D93" s="26" t="n"/>
       <c r="E93" s="26" t="n"/>
       <c r="F93" s="26" t="n"/>
-      <c r="G93" s="86" t="n"/>
-      <c r="H93" s="87" t="n"/>
-      <c r="I93" s="87" t="n"/>
-      <c r="J93" s="87" t="n"/>
+      <c r="G93" s="82" t="n"/>
+      <c r="H93" s="83" t="n"/>
+      <c r="I93" s="83" t="n"/>
+      <c r="J93" s="83" t="n"/>
     </row>
     <row r="94">
       <c r="B94" s="6" t="inlineStr">
@@ -3880,10 +3911,10 @@
       <c r="D94" s="26" t="n"/>
       <c r="E94" s="26" t="n"/>
       <c r="F94" s="26" t="n"/>
-      <c r="G94" s="88" t="n"/>
-      <c r="H94" s="87" t="n"/>
-      <c r="I94" s="87" t="n"/>
-      <c r="J94" s="87" t="n"/>
+      <c r="G94" s="84" t="n"/>
+      <c r="H94" s="83" t="n"/>
+      <c r="I94" s="83" t="n"/>
+      <c r="J94" s="83" t="n"/>
     </row>
     <row r="95">
       <c r="B95" s="6" t="inlineStr">
@@ -3897,16 +3928,16 @@
       <c r="D95" s="26" t="n"/>
       <c r="E95" s="26" t="n"/>
       <c r="F95" s="26" t="n"/>
-      <c r="G95" s="89" t="n"/>
-      <c r="H95" s="87" t="n"/>
-      <c r="I95" s="87" t="n"/>
-      <c r="J95" s="87" t="n"/>
+      <c r="G95" s="85" t="n"/>
+      <c r="H95" s="83" t="n"/>
+      <c r="I95" s="83" t="n"/>
+      <c r="J95" s="83" t="n"/>
     </row>
     <row r="96">
-      <c r="G96" s="90" t="n"/>
-      <c r="H96" s="91" t="n"/>
-      <c r="I96" s="91" t="n"/>
-      <c r="J96" s="91" t="n"/>
+      <c r="G96" s="86" t="n"/>
+      <c r="H96" s="87" t="n"/>
+      <c r="I96" s="87" t="n"/>
+      <c r="J96" s="87" t="n"/>
     </row>
     <row r="97">
       <c r="B97" s="11" t="inlineStr">
@@ -3934,10 +3965,10 @@
           <t>€ pro Jahr</t>
         </is>
       </c>
-      <c r="G97" s="92" t="n"/>
-      <c r="H97" s="93" t="n"/>
-      <c r="I97" s="93" t="n"/>
-      <c r="J97" s="93" t="n"/>
+      <c r="G97" s="88" t="n"/>
+      <c r="H97" s="89" t="n"/>
+      <c r="I97" s="89" t="n"/>
+      <c r="J97" s="89" t="n"/>
     </row>
     <row r="98">
       <c r="B98" s="2" t="inlineStr">
@@ -3959,10 +3990,10 @@
         <f>+E98*12</f>
         <v/>
       </c>
-      <c r="G98" s="94" t="n"/>
-      <c r="H98" s="95" t="n"/>
-      <c r="I98" s="96" t="n"/>
-      <c r="J98" s="96" t="n"/>
+      <c r="G98" s="90" t="n"/>
+      <c r="H98" s="91" t="n"/>
+      <c r="I98" s="92" t="n"/>
+      <c r="J98" s="92" t="n"/>
     </row>
     <row r="99">
       <c r="B99" s="6" t="inlineStr">
@@ -3985,10 +4016,10 @@
         <f>+E99*12</f>
         <v/>
       </c>
-      <c r="G99" s="97" t="n"/>
-      <c r="H99" s="98" t="n"/>
-      <c r="I99" s="96" t="n"/>
-      <c r="J99" s="96" t="n"/>
+      <c r="G99" s="93" t="n"/>
+      <c r="H99" s="94" t="n"/>
+      <c r="I99" s="92" t="n"/>
+      <c r="J99" s="92" t="n"/>
     </row>
     <row r="100">
       <c r="B100" s="6" t="inlineStr">
@@ -4010,10 +4041,10 @@
         <f>+E100*12</f>
         <v/>
       </c>
-      <c r="G100" s="99" t="n"/>
-      <c r="H100" s="98" t="n"/>
-      <c r="I100" s="96" t="n"/>
-      <c r="J100" s="96" t="n"/>
+      <c r="G100" s="95" t="n"/>
+      <c r="H100" s="94" t="n"/>
+      <c r="I100" s="92" t="n"/>
+      <c r="J100" s="92" t="n"/>
     </row>
     <row r="101">
       <c r="B101" s="6" t="inlineStr">
@@ -4035,10 +4066,10 @@
         <f>+E101*12</f>
         <v/>
       </c>
-      <c r="G101" s="97" t="n"/>
-      <c r="H101" s="98" t="n"/>
-      <c r="I101" s="96" t="n"/>
-      <c r="J101" s="96" t="n"/>
+      <c r="G101" s="93" t="n"/>
+      <c r="H101" s="94" t="n"/>
+      <c r="I101" s="92" t="n"/>
+      <c r="J101" s="92" t="n"/>
     </row>
     <row r="102">
       <c r="B102" s="6" t="inlineStr">
@@ -4060,10 +4091,10 @@
         <f>+E102*12</f>
         <v/>
       </c>
-      <c r="G102" s="97" t="n"/>
-      <c r="H102" s="98" t="n"/>
-      <c r="I102" s="96" t="n"/>
-      <c r="J102" s="96" t="n"/>
+      <c r="G102" s="93" t="n"/>
+      <c r="H102" s="94" t="n"/>
+      <c r="I102" s="92" t="n"/>
+      <c r="J102" s="92" t="n"/>
     </row>
     <row r="103">
       <c r="B103" s="6" t="inlineStr">
@@ -4085,10 +4116,10 @@
         <f>+E103*12</f>
         <v/>
       </c>
-      <c r="G103" s="99" t="n"/>
-      <c r="H103" s="98" t="n"/>
-      <c r="I103" s="96" t="n"/>
-      <c r="J103" s="96" t="n"/>
+      <c r="G103" s="95" t="n"/>
+      <c r="H103" s="94" t="n"/>
+      <c r="I103" s="92" t="n"/>
+      <c r="J103" s="92" t="n"/>
     </row>
     <row r="104" ht="8.25" customHeight="1">
       <c r="B104" s="14" t="n"/>
@@ -4096,10 +4127,10 @@
       <c r="D104" s="16" t="n"/>
       <c r="E104" s="17" t="n"/>
       <c r="F104" s="17" t="n"/>
-      <c r="G104" s="100" t="n"/>
-      <c r="H104" s="101" t="n"/>
-      <c r="I104" s="102" t="n"/>
-      <c r="J104" s="102" t="n"/>
+      <c r="G104" s="96" t="n"/>
+      <c r="H104" s="97" t="n"/>
+      <c r="I104" s="98" t="n"/>
+      <c r="J104" s="98" t="n"/>
     </row>
     <row r="105" customFormat="1" s="1">
       <c r="B105" s="1" t="inlineStr">
@@ -4117,10 +4148,10 @@
         <f>+SUM(F98:F104)</f>
         <v/>
       </c>
-      <c r="G105" s="103" t="n"/>
-      <c r="H105" s="104" t="n"/>
-      <c r="I105" s="105" t="n"/>
-      <c r="J105" s="105" t="n"/>
+      <c r="G105" s="99" t="n"/>
+      <c r="H105" s="100" t="n"/>
+      <c r="I105" s="101" t="n"/>
+      <c r="J105" s="101" t="n"/>
     </row>
     <row r="106" ht="6.75" customHeight="1" thickBot="1">
       <c r="B106" s="7" t="n"/>
@@ -4189,35 +4220,35 @@
           <t>Nettokaltmiete</t>
         </is>
       </c>
-      <c r="C109" s="126">
+      <c r="C109" s="109">
         <f>+C62+C80+C98</f>
         <v/>
       </c>
-      <c r="D109" s="127">
+      <c r="D109" s="110">
         <f>+IFERROR(E109/C109,0)</f>
         <v/>
       </c>
-      <c r="E109" s="128">
+      <c r="E109" s="111">
         <f>+E62+E80+E98</f>
         <v/>
       </c>
-      <c r="F109" s="128">
+      <c r="F109" s="111">
         <f>+E109*12</f>
         <v/>
       </c>
-      <c r="G109" s="129">
+      <c r="G109" s="112">
         <f>+G62+G80+G98</f>
         <v/>
       </c>
-      <c r="H109" s="127">
+      <c r="H109" s="110">
         <f>+IFERROR(I109/G109,0)</f>
         <v/>
       </c>
-      <c r="I109" s="128">
+      <c r="I109" s="111">
         <f>+I62+I80+I98</f>
         <v/>
       </c>
-      <c r="J109" s="128">
+      <c r="J109" s="111">
         <f>+I109*12</f>
         <v/>
       </c>
@@ -4228,35 +4259,35 @@
           <t>Nebenkostenpauschale</t>
         </is>
       </c>
-      <c r="C110" s="126">
+      <c r="C110" s="109">
         <f>+C63+C81+C99</f>
         <v/>
       </c>
-      <c r="D110" s="127">
+      <c r="D110" s="110">
         <f>+IFERROR(E110/C110,0)</f>
         <v/>
       </c>
-      <c r="E110" s="128">
+      <c r="E110" s="111">
         <f>+E63+E81+E99</f>
         <v/>
       </c>
-      <c r="F110" s="128">
+      <c r="F110" s="111">
         <f>+E110*12</f>
         <v/>
       </c>
-      <c r="G110" s="129">
+      <c r="G110" s="112">
         <f>+G63+G81+G99</f>
         <v/>
       </c>
-      <c r="H110" s="127">
+      <c r="H110" s="110">
         <f>+IFERROR(I110/G110,0)</f>
         <v/>
       </c>
-      <c r="I110" s="128">
+      <c r="I110" s="111">
         <f>+I63+I81+I99</f>
         <v/>
       </c>
-      <c r="J110" s="128">
+      <c r="J110" s="111">
         <f>+I110*12</f>
         <v/>
       </c>
@@ -4267,35 +4298,35 @@
           <t>Stellplätze</t>
         </is>
       </c>
-      <c r="C111" s="126">
+      <c r="C111" s="109">
         <f>+C64+C82+C100</f>
         <v/>
       </c>
-      <c r="D111" s="127">
+      <c r="D111" s="110">
         <f>+IFERROR(E111/C111,0)</f>
         <v/>
       </c>
-      <c r="E111" s="128">
+      <c r="E111" s="111">
         <f>+E64+E82+E100</f>
         <v/>
       </c>
-      <c r="F111" s="128">
+      <c r="F111" s="111">
         <f>+E111*12</f>
         <v/>
       </c>
-      <c r="G111" s="129">
+      <c r="G111" s="112">
         <f>+G64+G82+G100</f>
         <v/>
       </c>
-      <c r="H111" s="127">
+      <c r="H111" s="110">
         <f>+IFERROR(I111/G111,0)</f>
         <v/>
       </c>
-      <c r="I111" s="128">
+      <c r="I111" s="111">
         <f>+I64+I82+I100</f>
         <v/>
       </c>
-      <c r="J111" s="128">
+      <c r="J111" s="111">
         <f>+I111*12</f>
         <v/>
       </c>
@@ -4306,35 +4337,35 @@
           <t>Terasse</t>
         </is>
       </c>
-      <c r="C112" s="126">
+      <c r="C112" s="109">
         <f>+C65+C83+C101</f>
         <v/>
       </c>
-      <c r="D112" s="127">
+      <c r="D112" s="110">
         <f>+IFERROR(E112/C112,0)</f>
         <v/>
       </c>
-      <c r="E112" s="128">
+      <c r="E112" s="111">
         <f>+E65+E83+E101</f>
         <v/>
       </c>
-      <c r="F112" s="128">
+      <c r="F112" s="111">
         <f>+E112*12</f>
         <v/>
       </c>
-      <c r="G112" s="129">
+      <c r="G112" s="112">
         <f>+G65+G83+G101</f>
         <v/>
       </c>
-      <c r="H112" s="127">
+      <c r="H112" s="110">
         <f>+IFERROR(I112/G112,0)</f>
         <v/>
       </c>
-      <c r="I112" s="128">
+      <c r="I112" s="111">
         <f>+I65+I83+I101</f>
         <v/>
       </c>
-      <c r="J112" s="128">
+      <c r="J112" s="111">
         <f>+I112*12</f>
         <v/>
       </c>
@@ -4345,35 +4376,35 @@
           <t>Keller</t>
         </is>
       </c>
-      <c r="C113" s="126">
+      <c r="C113" s="109">
         <f>+C66+C84+C102</f>
         <v/>
       </c>
-      <c r="D113" s="127">
+      <c r="D113" s="110">
         <f>+IFERROR(E113/C113,0)</f>
         <v/>
       </c>
-      <c r="E113" s="128">
+      <c r="E113" s="111">
         <f>+E66+E84+E102</f>
         <v/>
       </c>
-      <c r="F113" s="128">
+      <c r="F113" s="111">
         <f>+E113*12</f>
         <v/>
       </c>
-      <c r="G113" s="129">
+      <c r="G113" s="112">
         <f>+G66+G84+G102</f>
         <v/>
       </c>
-      <c r="H113" s="127">
+      <c r="H113" s="110">
         <f>+IFERROR(I113/G113,0)</f>
         <v/>
       </c>
-      <c r="I113" s="128">
+      <c r="I113" s="111">
         <f>+I66+I84+I102</f>
         <v/>
       </c>
-      <c r="J113" s="128">
+      <c r="J113" s="111">
         <f>+I113*12</f>
         <v/>
       </c>
@@ -4384,35 +4415,35 @@
           <t>Sonstiges</t>
         </is>
       </c>
-      <c r="C114" s="126">
+      <c r="C114" s="109">
         <f>+C67+C85+C103</f>
         <v/>
       </c>
-      <c r="D114" s="127">
+      <c r="D114" s="110">
         <f>+IFERROR(E114/C114,0)</f>
         <v/>
       </c>
-      <c r="E114" s="128">
+      <c r="E114" s="111">
         <f>+E67+E85+E103</f>
         <v/>
       </c>
-      <c r="F114" s="128">
+      <c r="F114" s="111">
         <f>+E114*12</f>
         <v/>
       </c>
-      <c r="G114" s="129">
+      <c r="G114" s="112">
         <f>+G67+G85+G103</f>
         <v/>
       </c>
-      <c r="H114" s="127">
+      <c r="H114" s="110">
         <f>+IFERROR(I114/G114,0)</f>
         <v/>
       </c>
-      <c r="I114" s="128">
+      <c r="I114" s="111">
         <f>+I67+I85+I103</f>
         <v/>
       </c>
-      <c r="J114" s="128">
+      <c r="J114" s="111">
         <f>+I114*12</f>
         <v/>
       </c>
@@ -4462,887 +4493,1306 @@
     <row r="117">
       <c r="G117" s="52" t="n"/>
     </row>
-    <row r="118">
-      <c r="B118" s="82" t="inlineStr">
+    <row r="120" hidden="1" outlineLevel="1"/>
+    <row r="121" hidden="1" outlineLevel="1"/>
+    <row r="122" hidden="1" outlineLevel="1"/>
+    <row r="123" hidden="1" outlineLevel="1"/>
+    <row r="124" hidden="1" outlineLevel="1"/>
+    <row r="125" hidden="1" outlineLevel="1"/>
+    <row r="126" hidden="1" outlineLevel="1"/>
+    <row r="127" hidden="1" outlineLevel="1"/>
+    <row r="128" hidden="1" outlineLevel="1"/>
+    <row r="129" hidden="1" outlineLevel="1">
+      <c r="L129" s="47" t="n"/>
+    </row>
+    <row r="130" hidden="1" outlineLevel="1"/>
+    <row r="131" hidden="1" outlineLevel="1"/>
+    <row r="132" hidden="1" outlineLevel="1" ht="8.25" customHeight="1"/>
+    <row r="133" hidden="1" outlineLevel="1" customFormat="1" s="1"/>
+    <row r="134" hidden="1" outlineLevel="1" ht="6.75" customHeight="1"/>
+    <row r="135" hidden="1" outlineLevel="1" ht="6.75" customHeight="1"/>
+    <row r="136" hidden="1" outlineLevel="1"/>
+    <row r="137" hidden="1" outlineLevel="1"/>
+    <row r="138" hidden="1" outlineLevel="1"/>
+    <row r="139" hidden="1" outlineLevel="1" ht="6.75" customHeight="1"/>
+    <row r="140" hidden="1" outlineLevel="1"/>
+    <row r="141" hidden="1" outlineLevel="1"/>
+    <row r="142" hidden="1" outlineLevel="1"/>
+    <row r="143" hidden="1" outlineLevel="1"/>
+    <row r="144" hidden="1" outlineLevel="1"/>
+    <row r="145" hidden="1" outlineLevel="1"/>
+    <row r="146" hidden="1" outlineLevel="1"/>
+    <row r="147" hidden="1" outlineLevel="1"/>
+    <row r="148" hidden="1" outlineLevel="1"/>
+    <row r="149" hidden="1" outlineLevel="1"/>
+    <row r="150" hidden="1" outlineLevel="1"/>
+    <row r="151" hidden="1" outlineLevel="1"/>
+    <row r="152" hidden="1" outlineLevel="1"/>
+    <row r="153" hidden="1" outlineLevel="1" ht="8.25" customHeight="1"/>
+    <row r="154" hidden="1" outlineLevel="1" customFormat="1" s="1"/>
+    <row r="155" hidden="1" outlineLevel="1" ht="6.75" customHeight="1"/>
+    <row r="156" hidden="1" outlineLevel="1"/>
+    <row r="157" collapsed="1"/>
+    <row r="158">
+      <c r="B158" s="78" t="inlineStr">
         <is>
           <t>Berechnung Indexklausel - laut Vermieter beträgt die angepasste Miete 14,95 Euro</t>
         </is>
       </c>
-      <c r="G118" s="52" t="n"/>
-    </row>
-    <row r="119">
-      <c r="B119" s="6" t="inlineStr">
-        <is>
-          <t>Nettokaltmiete bisher (€/qm)</t>
-        </is>
-      </c>
-      <c r="C119" s="121" t="n">
+      <c r="G158" s="126" t="n"/>
+    </row>
+    <row r="159">
+      <c r="B159" s="6" t="n"/>
+      <c r="C159" s="104" t="n"/>
+    </row>
+    <row r="160">
+      <c r="B160" s="127" t="inlineStr">
+        <is>
+          <t>Referenzwerte VPI Deutschland (Destatis, Basis 2020 = 100)</t>
+        </is>
+      </c>
+      <c r="C160" s="104" t="n"/>
+    </row>
+    <row r="161">
+      <c r="B161" s="128" t="inlineStr">
+        <is>
+          <t>VPI 04/2021 – Basis: Flächen 2./3. + 4. OG, 9 Stellplätze</t>
+        </is>
+      </c>
+      <c r="C161" s="129" t="n">
+        <v>102.4</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="B162" s="128" t="inlineStr">
+        <is>
+          <t>VPI 04/2022 – Basis: Keller Nr. 09, 2 Stellplätze</t>
+        </is>
+      </c>
+      <c r="C162" s="129" t="n">
+        <v>108.8</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="B163" s="128" t="inlineStr">
+        <is>
+          <t>VPI 04/2023 – Basis: Keller 70 qm</t>
+        </is>
+      </c>
+      <c r="C163" s="129" t="n">
+        <v>116.6</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="B164" s="128" t="inlineStr">
+        <is>
+          <t>VPI 10/2023 – Basis: 1. OG, 3 Stellplätze</t>
+        </is>
+      </c>
+      <c r="C164" s="129" t="n">
+        <v>117.8</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="B165" s="128" t="inlineStr">
+        <is>
+          <t>VPI Referenzmonat (hier 04/2025, frühester Anpassungstermin)</t>
+        </is>
+      </c>
+      <c r="C165" s="129" t="n">
+        <v>121.7</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="B166" s="6" t="n"/>
+      <c r="C166" s="108" t="n"/>
+    </row>
+    <row r="167">
+      <c r="B167" s="130" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="C167" s="130" t="inlineStr">
+        <is>
+          <t>Menge</t>
+        </is>
+      </c>
+      <c r="D167" s="130" t="inlineStr">
+        <is>
+          <t>alt € / Einheit</t>
+        </is>
+      </c>
+      <c r="E167" s="130" t="inlineStr">
+        <is>
+          <t>Basis-VPI</t>
+        </is>
+      </c>
+      <c r="F167" s="130" t="inlineStr">
+        <is>
+          <t>Indexveränderung</t>
+        </is>
+      </c>
+      <c r="G167" s="130" t="inlineStr">
+        <is>
+          <t>zulässig € / Einheit</t>
+        </is>
+      </c>
+      <c r="H167" s="130" t="inlineStr">
+        <is>
+          <t>alt € / Monat</t>
+        </is>
+      </c>
+      <c r="I167" s="130" t="inlineStr">
+        <is>
+          <t>neu € / Monat</t>
+        </is>
+      </c>
+      <c r="J167" s="130" t="inlineStr">
+        <is>
+          <t>Differenz € / Monat</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="B168" s="128" t="inlineStr">
+        <is>
+          <t>Flächen 2./3. OG</t>
+        </is>
+      </c>
+      <c r="C168" s="131" t="n">
+        <v>695.28</v>
+      </c>
+      <c r="D168" s="104" t="n">
         <v>12.5</v>
       </c>
-    </row>
-    <row r="120" hidden="1" outlineLevel="1">
-      <c r="B120" s="6" t="inlineStr">
+      <c r="E168" s="132">
+        <f>+$C$161</f>
+        <v/>
+      </c>
+      <c r="F168" s="133">
+        <f>+$C$165/E168-1</f>
+        <v/>
+      </c>
+      <c r="G168" s="107">
+        <f>+IF(F168&gt;0.05,D168*(1+F168),D168)</f>
+        <v/>
+      </c>
+      <c r="H168" s="107">
+        <f>+C168*D168</f>
+        <v/>
+      </c>
+      <c r="I168" s="107">
+        <f>+C168*G168</f>
+        <v/>
+      </c>
+      <c r="J168" s="107">
+        <f>+I168-H168</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="B169" s="128" t="inlineStr">
+        <is>
+          <t>Fläche 4. OG</t>
+        </is>
+      </c>
+      <c r="C169" s="131" t="n">
+        <v>59</v>
+      </c>
+      <c r="D169" s="104" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E169" s="132">
+        <f>+$C$161</f>
+        <v/>
+      </c>
+      <c r="F169" s="133">
+        <f>+$C$165/E169-1</f>
+        <v/>
+      </c>
+      <c r="G169" s="107">
+        <f>+IF(F169&gt;0.05,D169*(1+F169),D169)</f>
+        <v/>
+      </c>
+      <c r="H169" s="107">
+        <f>+C169*D169</f>
+        <v/>
+      </c>
+      <c r="I169" s="107">
+        <f>+C169*G169</f>
+        <v/>
+      </c>
+      <c r="J169" s="107">
+        <f>+I169-H169</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" s="128" t="inlineStr">
+        <is>
+          <t>Fläche 1. OG</t>
+        </is>
+      </c>
+      <c r="C170" s="131" t="n">
+        <v>350.32</v>
+      </c>
+      <c r="D170" s="104" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E170" s="132">
+        <f>+$C$164</f>
+        <v/>
+      </c>
+      <c r="F170" s="133">
+        <f>+$C$165/E170-1</f>
+        <v/>
+      </c>
+      <c r="G170" s="107">
+        <f>+IF(F170&gt;0.05,D170*(1+F170),D170)</f>
+        <v/>
+      </c>
+      <c r="H170" s="107">
+        <f>+C170*D170</f>
+        <v/>
+      </c>
+      <c r="I170" s="107">
+        <f>+C170*G170</f>
+        <v/>
+      </c>
+      <c r="J170" s="107">
+        <f>+I170-H170</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" s="128" t="inlineStr">
+        <is>
+          <t>Keller Nr. 09</t>
+        </is>
+      </c>
+      <c r="C171" s="131" t="n">
+        <v>18.65</v>
+      </c>
+      <c r="D171" s="104" t="n">
+        <v>5</v>
+      </c>
+      <c r="E171" s="132">
+        <f>+$C$162</f>
+        <v/>
+      </c>
+      <c r="F171" s="133">
+        <f>+$C$165/E171-1</f>
+        <v/>
+      </c>
+      <c r="G171" s="107">
+        <f>+IF(F171&gt;0.05,D171*(1+F171),D171)</f>
+        <v/>
+      </c>
+      <c r="H171" s="107">
+        <f>+C171*D171</f>
+        <v/>
+      </c>
+      <c r="I171" s="107">
+        <f>+C171*G171</f>
+        <v/>
+      </c>
+      <c r="J171" s="107">
+        <f>+I171-H171</f>
+        <v/>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" s="128" t="inlineStr">
+        <is>
+          <t>Keller 70 qm</t>
+        </is>
+      </c>
+      <c r="C172" s="131" t="n">
+        <v>70</v>
+      </c>
+      <c r="D172" s="104" t="n">
+        <v>5</v>
+      </c>
+      <c r="E172" s="132">
+        <f>+$C$163</f>
+        <v/>
+      </c>
+      <c r="F172" s="133">
+        <f>+$C$165/E172-1</f>
+        <v/>
+      </c>
+      <c r="G172" s="107">
+        <f>+IF(F172&gt;0.05,D172*(1+F172),D172)</f>
+        <v/>
+      </c>
+      <c r="H172" s="107">
+        <f>+C172*D172</f>
+        <v/>
+      </c>
+      <c r="I172" s="107">
+        <f>+C172*G172</f>
+        <v/>
+      </c>
+      <c r="J172" s="107">
+        <f>+I172-H172</f>
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="B173" s="128" t="inlineStr">
+        <is>
+          <t>Stellplätze (ab 04/2021)</t>
+        </is>
+      </c>
+      <c r="C173" s="131" t="n">
+        <v>9</v>
+      </c>
+      <c r="D173" s="104" t="n">
+        <v>40</v>
+      </c>
+      <c r="E173" s="132">
+        <f>+$C$161</f>
+        <v/>
+      </c>
+      <c r="F173" s="133">
+        <f>+$C$165/E173-1</f>
+        <v/>
+      </c>
+      <c r="G173" s="107">
+        <f>+IF(F173&gt;0.05,D173*(1+F173),D173)</f>
+        <v/>
+      </c>
+      <c r="H173" s="107">
+        <f>+C173*D173</f>
+        <v/>
+      </c>
+      <c r="I173" s="107">
+        <f>+C173*G173</f>
+        <v/>
+      </c>
+      <c r="J173" s="107">
+        <f>+I173-H173</f>
+        <v/>
+      </c>
+    </row>
+    <row r="174">
+      <c r="B174" s="128" t="inlineStr">
+        <is>
+          <t>Stellplätze (ab 04/2022)</t>
+        </is>
+      </c>
+      <c r="C174" s="131" t="n">
+        <v>2</v>
+      </c>
+      <c r="D174" s="104" t="n">
+        <v>60</v>
+      </c>
+      <c r="E174" s="132">
+        <f>+$C$162</f>
+        <v/>
+      </c>
+      <c r="F174" s="133">
+        <f>+$C$165/E174-1</f>
+        <v/>
+      </c>
+      <c r="G174" s="107">
+        <f>+IF(F174&gt;0.05,D174*(1+F174),D174)</f>
+        <v/>
+      </c>
+      <c r="H174" s="107">
+        <f>+C174*D174</f>
+        <v/>
+      </c>
+      <c r="I174" s="107">
+        <f>+C174*G174</f>
+        <v/>
+      </c>
+      <c r="J174" s="107">
+        <f>+I174-H174</f>
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="B175" s="128" t="inlineStr">
+        <is>
+          <t>Stellplätze (ab 10/2023)</t>
+        </is>
+      </c>
+      <c r="C175" s="131" t="n">
+        <v>3</v>
+      </c>
+      <c r="D175" s="104" t="n">
+        <v>60</v>
+      </c>
+      <c r="E175" s="132">
+        <f>+$C$164</f>
+        <v/>
+      </c>
+      <c r="F175" s="133">
+        <f>+$C$165/E175-1</f>
+        <v/>
+      </c>
+      <c r="G175" s="107">
+        <f>+IF(F175&gt;0.05,D175*(1+F175),D175)</f>
+        <v/>
+      </c>
+      <c r="H175" s="107">
+        <f>+C175*D175</f>
+        <v/>
+      </c>
+      <c r="I175" s="107">
+        <f>+C175*G175</f>
+        <v/>
+      </c>
+      <c r="J175" s="107">
+        <f>+I175-H175</f>
+        <v/>
+      </c>
+    </row>
+    <row r="176">
+      <c r="B176" s="134" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="H176" s="135">
+        <f>+SUM(H168:H175)</f>
+        <v/>
+      </c>
+      <c r="I176" s="135">
+        <f>+SUM(I168:I175)</f>
+        <v/>
+      </c>
+      <c r="J176" s="135">
+        <f>+SUM(J168:J175)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="177"/>
+    <row r="178">
+      <c r="B178" s="128" t="inlineStr">
         <is>
           <t>Forderung Vermieter (€/qm)</t>
         </is>
       </c>
-      <c r="C120" s="121" t="n">
+      <c r="C178" s="104" t="n">
         <v>14.95</v>
       </c>
     </row>
-    <row r="121" hidden="1" outlineLevel="1">
-      <c r="B121" s="6" t="inlineStr">
-        <is>
-          <t>implizite Erhöhung</t>
-        </is>
-      </c>
-      <c r="C121" s="122">
-        <f>+C120/C119-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="122" hidden="1" outlineLevel="1">
-      <c r="B122" s="6" t="inlineStr">
-        <is>
-          <t>VPI 04/2021 – Basis 2./3. + 4. OG (Destatis)</t>
-        </is>
-      </c>
-      <c r="C122" s="123" t="n">
-        <v>102.4</v>
-      </c>
-    </row>
-    <row r="123" hidden="1" outlineLevel="1">
-      <c r="B123" s="6" t="inlineStr">
-        <is>
-          <t>VPI 04/2025 – frühester Anpassungstermin (Destatis)</t>
-        </is>
-      </c>
-      <c r="C123" s="123" t="n">
-        <v>121.7</v>
-      </c>
-    </row>
-    <row r="124" hidden="1" outlineLevel="1">
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>tatsächliche Indexveränderung</t>
-        </is>
-      </c>
-      <c r="C124" s="122">
-        <f>+IFERROR(C123/C122-1,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="125" hidden="1" outlineLevel="1">
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>zulässige Miete rechnerisch (€/qm)</t>
-        </is>
-      </c>
-      <c r="C125" s="124">
-        <f>+IFERROR(C119*C123/C122,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="126" hidden="1" outlineLevel="1">
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>Basis 1. OG: VPI 10/2023 = 117,8 → nur +3,31 %, unter der 5 %-Schwelle</t>
-        </is>
-      </c>
-      <c r="C126" s="125" t="n"/>
-    </row>
-    <row r="127" hidden="1" outlineLevel="1">
-      <c r="B127" s="6" t="inlineStr">
-        <is>
-          <t>VPI 07/2026 – aktueller Stand (Destatis)</t>
-        </is>
-      </c>
-      <c r="C127" s="123" t="n">
-        <v>125.6</v>
-      </c>
-      <c r="G127" s="52" t="n"/>
-    </row>
-    <row r="128" hidden="1" outlineLevel="1">
-      <c r="B128" s="23" t="inlineStr">
+    <row r="179">
+      <c r="B179" s="128" t="inlineStr">
+        <is>
+          <t>implizite Erhöhung gegenüber 12,50 €</t>
+        </is>
+      </c>
+      <c r="C179" s="133">
+        <f>+C178/D168-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="180">
+      <c r="B180" s="128" t="inlineStr">
+        <is>
+          <t>Nettokaltmiete Flächen nach Forderung (€/Monat)</t>
+        </is>
+      </c>
+      <c r="C180" s="107">
+        <f>+(C168+C169+C170)*C178</f>
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="B181" s="128" t="inlineStr">
+        <is>
+          <t>davon nicht durch die Indexklausel gedeckt (€/Monat)</t>
+        </is>
+      </c>
+      <c r="C181" s="135">
+        <f>+C180-(I168+I169+I170)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="182" ht="15.75" customHeight="1" thickBot="1">
+      <c r="B182" s="23" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="C128" s="23" t="inlineStr">
+      <c r="C182" s="23" t="inlineStr">
         <is>
           <t>Anmerkungen</t>
         </is>
       </c>
-      <c r="D128" s="24" t="n"/>
-      <c r="E128" s="24" t="n"/>
-      <c r="F128" s="24" t="n"/>
-      <c r="G128" s="69" t="inlineStr">
+      <c r="D182" s="24" t="n"/>
+      <c r="E182" s="24" t="n"/>
+      <c r="F182" s="24" t="n"/>
+      <c r="G182" s="69" t="inlineStr">
         <is>
           <t>Anmerkungen</t>
         </is>
       </c>
-      <c r="H128" s="24" t="n"/>
-      <c r="I128" s="24" t="n"/>
-      <c r="J128" s="24" t="n"/>
-    </row>
-    <row r="129" hidden="1" outlineLevel="1">
-      <c r="B129" s="35" t="inlineStr">
+      <c r="H182" s="24" t="n"/>
+      <c r="I182" s="24" t="n"/>
+      <c r="J182" s="24" t="n"/>
+    </row>
+    <row r="183">
+      <c r="B183" s="35" t="inlineStr">
         <is>
           <t>Möbel Patientenzimmer</t>
         </is>
       </c>
-      <c r="C129" s="36" t="inlineStr">
+      <c r="C183" s="36" t="inlineStr">
         <is>
           <t>Mieter</t>
         </is>
       </c>
-      <c r="D129" s="37" t="n"/>
-      <c r="E129" s="38" t="n"/>
-      <c r="F129" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G129" s="70" t="inlineStr">
+      <c r="D183" s="37" t="n"/>
+      <c r="E183" s="38" t="n"/>
+      <c r="F183" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G183" s="70" t="inlineStr">
         <is>
           <t>Pflegebetten im Inventar</t>
         </is>
       </c>
-      <c r="H129" s="37" t="n"/>
-      <c r="I129" s="38" t="n"/>
-      <c r="J129" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L129" s="47" t="n"/>
-    </row>
-    <row r="130" hidden="1" outlineLevel="1">
-      <c r="B130" s="35" t="inlineStr">
+      <c r="H183" s="37" t="n"/>
+      <c r="I183" s="38" t="n"/>
+      <c r="J183" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="B184" s="35" t="inlineStr">
         <is>
           <t>Gemeinschaftsbereich</t>
         </is>
       </c>
-      <c r="C130" s="25" t="inlineStr">
+      <c r="C184" s="25" t="inlineStr">
         <is>
           <t>Mieter</t>
         </is>
       </c>
-      <c r="D130" s="39" t="n"/>
-      <c r="E130" s="40" t="n"/>
-      <c r="F130" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G130" s="54" t="inlineStr">
+      <c r="D184" s="39" t="n"/>
+      <c r="E184" s="40" t="n"/>
+      <c r="F184" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G184" s="54" t="inlineStr">
         <is>
           <t>Einbauküchen, Vorhänge im Inventar</t>
         </is>
       </c>
-      <c r="H130" s="39" t="n"/>
-      <c r="I130" s="40" t="n"/>
-      <c r="J130" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131" hidden="1" outlineLevel="1">
-      <c r="B131" s="35" t="inlineStr">
+      <c r="H184" s="39" t="n"/>
+      <c r="I184" s="40" t="n"/>
+      <c r="J184" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="B185" s="35" t="inlineStr">
         <is>
           <t>Schwesternrufanlage</t>
         </is>
       </c>
-      <c r="C131" s="25" t="inlineStr">
+      <c r="C185" s="25" t="inlineStr">
         <is>
           <t>Mieter</t>
         </is>
       </c>
-      <c r="D131" s="39" t="n"/>
-      <c r="E131" s="40" t="n"/>
-      <c r="F131" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G131" s="54" t="inlineStr">
+      <c r="D185" s="39" t="n"/>
+      <c r="E185" s="40" t="n"/>
+      <c r="F185" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G185" s="54" t="inlineStr">
         <is>
           <t>vorhanden; Unterhaltung als Nebenkosten</t>
         </is>
       </c>
-      <c r="H131" s="39" t="n"/>
-      <c r="I131" s="40" t="n"/>
-      <c r="J131" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" hidden="1" outlineLevel="1" ht="8.25" customHeight="1">
-      <c r="B132" s="35" t="inlineStr">
+      <c r="H185" s="39" t="n"/>
+      <c r="I185" s="40" t="n"/>
+      <c r="J185" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="B186" s="35" t="inlineStr">
         <is>
           <t>Pflegebad</t>
         </is>
       </c>
-      <c r="C132" s="25" t="inlineStr">
+      <c r="C186" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D132" s="39" t="n"/>
-      <c r="E132" s="40" t="n"/>
-      <c r="F132" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G132" s="54" t="inlineStr">
+      <c r="D186" s="39" t="n"/>
+      <c r="E186" s="40" t="n"/>
+      <c r="F186" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G186" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H132" s="39" t="n"/>
-      <c r="I132" s="40" t="n"/>
-      <c r="J132" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133" hidden="1" outlineLevel="1" customFormat="1" s="1">
-      <c r="B133" s="35" t="inlineStr">
+      <c r="H186" s="39" t="n"/>
+      <c r="I186" s="40" t="n"/>
+      <c r="J186" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" ht="15.75" customHeight="1" thickBot="1">
+      <c r="B187" s="35" t="inlineStr">
         <is>
           <t>Fäkalienspüle</t>
         </is>
       </c>
-      <c r="C133" s="25" t="inlineStr">
+      <c r="C187" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D133" s="39" t="n"/>
-      <c r="E133" s="40" t="n"/>
-      <c r="F133" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G133" s="54" t="inlineStr">
+      <c r="D187" s="39" t="n"/>
+      <c r="E187" s="40" t="n"/>
+      <c r="F187" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G187" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H133" s="39" t="n"/>
-      <c r="I133" s="40" t="n"/>
-      <c r="J133" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134" hidden="1" outlineLevel="1" ht="6.75" customHeight="1" thickBot="1">
-      <c r="B134" s="35" t="inlineStr">
+      <c r="H187" s="39" t="n"/>
+      <c r="I187" s="40" t="n"/>
+      <c r="J187" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="B188" s="35" t="inlineStr">
         <is>
           <t>Umbaukosten</t>
         </is>
       </c>
-      <c r="C134" s="25" t="inlineStr">
+      <c r="C188" s="25" t="inlineStr">
         <is>
           <t>Vermieter baut aus; Sonderwünsche zu Lasten Mieter</t>
         </is>
       </c>
-      <c r="D134" s="39" t="n"/>
-      <c r="E134" s="40" t="n"/>
-      <c r="F134" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G134" s="54" t="inlineStr">
+      <c r="D188" s="39" t="n"/>
+      <c r="E188" s="40" t="n"/>
+      <c r="F188" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G188" s="54" t="inlineStr">
         <is>
           <t>kein Umbau - laufender Betrieb übernommen</t>
         </is>
       </c>
-      <c r="H134" s="39" t="n"/>
-      <c r="I134" s="40" t="n"/>
-      <c r="J134" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" hidden="1" outlineLevel="1" ht="6.75" customHeight="1">
-      <c r="B135" s="35" t="inlineStr">
+      <c r="H188" s="39" t="n"/>
+      <c r="I188" s="40" t="n"/>
+      <c r="J188" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="B189" s="35" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="C135" s="25" t="inlineStr">
+      <c r="C189" s="25" t="inlineStr">
         <is>
           <t>Mieter</t>
         </is>
       </c>
-      <c r="D135" s="39" t="n"/>
-      <c r="E135" s="40" t="n"/>
-      <c r="F135" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G135" s="54" t="inlineStr">
+      <c r="D189" s="39" t="n"/>
+      <c r="E189" s="40" t="n"/>
+      <c r="F189" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G189" s="54" t="inlineStr">
         <is>
           <t>Mieter</t>
         </is>
       </c>
-      <c r="H135" s="39" t="n"/>
-      <c r="I135" s="40" t="n"/>
-      <c r="J135" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" hidden="1" outlineLevel="1">
-      <c r="B136" s="35" t="inlineStr">
+      <c r="H189" s="39" t="n"/>
+      <c r="I189" s="40" t="n"/>
+      <c r="J189" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="B190" s="35" t="inlineStr">
         <is>
           <t>Waschmaschinen</t>
         </is>
       </c>
-      <c r="C136" s="25" t="inlineStr">
+      <c r="C190" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D136" s="39" t="n"/>
-      <c r="E136" s="40" t="n"/>
-      <c r="F136" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G136" s="54" t="inlineStr">
+      <c r="D190" s="39" t="n"/>
+      <c r="E190" s="40" t="n"/>
+      <c r="F190" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G190" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H136" s="39" t="n"/>
-      <c r="I136" s="40" t="n"/>
-      <c r="J136" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" hidden="1" outlineLevel="1">
-      <c r="B137" s="35" t="inlineStr">
+      <c r="H190" s="39" t="n"/>
+      <c r="I190" s="40" t="n"/>
+      <c r="J190" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="B191" s="35" t="inlineStr">
         <is>
           <t>[Platzhalter]</t>
         </is>
       </c>
-      <c r="C137" s="25" t="inlineStr">
+      <c r="C191" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D137" s="39" t="n"/>
-      <c r="E137" s="40" t="n"/>
-      <c r="F137" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G137" s="54" t="inlineStr">
+      <c r="D191" s="39" t="n"/>
+      <c r="E191" s="40" t="n"/>
+      <c r="F191" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G191" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H137" s="39" t="n"/>
-      <c r="I137" s="40" t="n"/>
-      <c r="J137" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" hidden="1" outlineLevel="1">
-      <c r="B138" s="35" t="inlineStr">
+      <c r="H191" s="39" t="n"/>
+      <c r="I191" s="40" t="n"/>
+      <c r="J191" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="B192" s="35" t="inlineStr">
         <is>
           <t>[Platzhalter]</t>
         </is>
       </c>
-      <c r="C138" s="25" t="inlineStr">
+      <c r="C192" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D138" s="39" t="n"/>
-      <c r="E138" s="40" t="n"/>
-      <c r="F138" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G138" s="54" t="inlineStr">
+      <c r="D192" s="39" t="n"/>
+      <c r="E192" s="40" t="n"/>
+      <c r="F192" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G192" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H138" s="39" t="n"/>
-      <c r="I138" s="40" t="n"/>
-      <c r="J138" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" hidden="1" outlineLevel="1" ht="6.75" customHeight="1" thickBot="1">
-      <c r="B139" s="35" t="inlineStr">
+      <c r="H192" s="39" t="n"/>
+      <c r="I192" s="40" t="n"/>
+      <c r="J192" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="B193" s="35" t="inlineStr">
         <is>
           <t>[Platzhalter]</t>
         </is>
       </c>
-      <c r="C139" s="25" t="inlineStr">
+      <c r="C193" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D139" s="39" t="n"/>
-      <c r="E139" s="40" t="n"/>
-      <c r="F139" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G139" s="54" t="inlineStr">
+      <c r="D193" s="39" t="n"/>
+      <c r="E193" s="40" t="n"/>
+      <c r="F193" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G193" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H139" s="39" t="n"/>
-      <c r="I139" s="40" t="n"/>
-      <c r="J139" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140" hidden="1" outlineLevel="1">
-      <c r="B140" s="14" t="n"/>
-      <c r="C140" s="15" t="n"/>
-      <c r="D140" s="16" t="n"/>
-      <c r="E140" s="17" t="n"/>
-      <c r="F140" s="17" t="n"/>
-      <c r="G140" s="67" t="n"/>
-      <c r="H140" s="16" t="n"/>
-      <c r="I140" s="17" t="n"/>
-      <c r="J140" s="17" t="n"/>
-    </row>
-    <row r="141" hidden="1" outlineLevel="1">
-      <c r="B141" s="1" t="inlineStr">
+      <c r="H193" s="39" t="n"/>
+      <c r="I193" s="40" t="n"/>
+      <c r="J193" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="B194" s="14" t="n"/>
+      <c r="C194" s="15" t="n"/>
+      <c r="D194" s="16" t="n"/>
+      <c r="E194" s="17" t="n"/>
+      <c r="F194" s="17" t="n"/>
+      <c r="G194" s="67" t="n"/>
+      <c r="H194" s="16" t="n"/>
+      <c r="I194" s="17" t="n"/>
+      <c r="J194" s="17" t="n"/>
+    </row>
+    <row r="195">
+      <c r="B195" s="1" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="C141" s="18" t="n"/>
-      <c r="D141" s="19" t="n"/>
-      <c r="E141" s="20" t="n"/>
-      <c r="F141" s="20">
-        <f>+SUM(F129:F140)</f>
-        <v/>
-      </c>
-      <c r="G141" s="68" t="n"/>
-      <c r="H141" s="19" t="n"/>
-      <c r="I141" s="20" t="n"/>
-      <c r="J141" s="20">
-        <f>+SUM(J129:J140)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="142" hidden="1" outlineLevel="1">
-      <c r="B142" s="7" t="n"/>
-      <c r="C142" s="8" t="n"/>
-      <c r="D142" s="7" t="n"/>
-      <c r="E142" s="7" t="n"/>
-      <c r="F142" s="7" t="n"/>
-      <c r="G142" s="55" t="n"/>
-      <c r="H142" s="7" t="n"/>
-      <c r="I142" s="7" t="n"/>
-      <c r="J142" s="7" t="n"/>
-    </row>
-    <row r="143" hidden="1" outlineLevel="1">
-      <c r="G143" s="52" t="n"/>
-    </row>
-    <row r="144" hidden="1" outlineLevel="1">
-      <c r="B144" s="21" t="inlineStr">
+      <c r="C195" s="18" t="n"/>
+      <c r="D195" s="19" t="n"/>
+      <c r="E195" s="20" t="n"/>
+      <c r="F195" s="20">
+        <f>+SUM(F183:F194)</f>
+        <v/>
+      </c>
+      <c r="G195" s="68" t="n"/>
+      <c r="H195" s="19" t="n"/>
+      <c r="I195" s="20" t="n"/>
+      <c r="J195" s="20">
+        <f>+SUM(J183:J194)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="B196" s="7" t="n"/>
+      <c r="C196" s="8" t="n"/>
+      <c r="D196" s="7" t="n"/>
+      <c r="E196" s="7" t="n"/>
+      <c r="F196" s="7" t="n"/>
+      <c r="G196" s="55" t="n"/>
+      <c r="H196" s="7" t="n"/>
+      <c r="I196" s="7" t="n"/>
+      <c r="J196" s="7" t="n"/>
+    </row>
+    <row r="197">
+      <c r="G197" s="52" t="n"/>
+    </row>
+    <row r="198">
+      <c r="B198" s="21" t="inlineStr">
         <is>
           <t>davon:</t>
         </is>
       </c>
-      <c r="G144" s="52" t="n"/>
-    </row>
-    <row r="145" hidden="1" outlineLevel="1">
-      <c r="B145" s="22" t="inlineStr">
+      <c r="G198" s="52" t="n"/>
+    </row>
+    <row r="199">
+      <c r="B199" s="22" t="inlineStr">
         <is>
           <t>Übernahme Vermieter</t>
         </is>
       </c>
-      <c r="C145" s="25" t="inlineStr">
+      <c r="C199" s="25" t="inlineStr">
         <is>
           <t>Ausbau nach Raumbuch (liegt nicht vor)</t>
         </is>
       </c>
-      <c r="D145" s="39" t="n"/>
-      <c r="E145" s="40" t="n"/>
-      <c r="F145" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G145" s="54" t="inlineStr">
+      <c r="D199" s="39" t="n"/>
+      <c r="E199" s="40" t="n"/>
+      <c r="F199" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G199" s="54" t="inlineStr">
         <is>
           <t>Inventar durch Vermieterseite gestellt</t>
         </is>
       </c>
-      <c r="H145" s="39" t="n"/>
-      <c r="I145" s="40" t="n"/>
-      <c r="J145" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="146" hidden="1" outlineLevel="1">
-      <c r="B146" s="22" t="inlineStr">
+      <c r="H199" s="39" t="n"/>
+      <c r="I199" s="40" t="n"/>
+      <c r="J199" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="B200" s="22" t="inlineStr">
         <is>
           <t>Baukostenzuschuss Mieter</t>
         </is>
       </c>
-      <c r="C146" s="25" t="inlineStr">
+      <c r="C200" s="25" t="inlineStr">
         <is>
           <t>600€/Monat für Statik, 1. OG</t>
         </is>
       </c>
-      <c r="D146" s="39" t="n"/>
-      <c r="E146" s="40" t="n"/>
-      <c r="F146" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G146" s="54" t="inlineStr">
+      <c r="D200" s="39" t="n"/>
+      <c r="E200" s="40" t="n"/>
+      <c r="F200" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G200" s="54" t="inlineStr">
         <is>
           <t>Kein BKZ</t>
         </is>
       </c>
-      <c r="H146" s="39" t="n"/>
-      <c r="I146" s="40" t="n"/>
-      <c r="J146" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="147" hidden="1" outlineLevel="1">
-      <c r="B147" s="7" t="n"/>
-      <c r="C147" s="8" t="n"/>
-      <c r="D147" s="7" t="n"/>
-      <c r="E147" s="7" t="n"/>
-      <c r="F147" s="7" t="n"/>
-      <c r="G147" s="55" t="n"/>
-      <c r="H147" s="7" t="n"/>
-      <c r="I147" s="7" t="n"/>
-      <c r="J147" s="7" t="n"/>
-    </row>
-    <row r="148" hidden="1" outlineLevel="1">
-      <c r="G148" s="52" t="n"/>
-    </row>
-    <row r="149" hidden="1" outlineLevel="1">
-      <c r="G149" s="52" t="n"/>
-    </row>
-    <row r="150" hidden="1" outlineLevel="1">
-      <c r="B150" s="23" t="inlineStr">
+      <c r="H200" s="39" t="n"/>
+      <c r="I200" s="40" t="n"/>
+      <c r="J200" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="B201" s="7" t="n"/>
+      <c r="C201" s="8" t="n"/>
+      <c r="D201" s="7" t="n"/>
+      <c r="E201" s="7" t="n"/>
+      <c r="F201" s="7" t="n"/>
+      <c r="G201" s="55" t="n"/>
+      <c r="H201" s="7" t="n"/>
+      <c r="I201" s="7" t="n"/>
+      <c r="J201" s="7" t="n"/>
+    </row>
+    <row r="202">
+      <c r="G202" s="52" t="n"/>
+    </row>
+    <row r="203" ht="15.75" customHeight="1" thickBot="1">
+      <c r="G203" s="52" t="n"/>
+    </row>
+    <row r="204">
+      <c r="B204" s="23" t="inlineStr">
         <is>
           <t>Ramp-up Kosten</t>
         </is>
       </c>
-      <c r="C150" s="23" t="inlineStr">
+      <c r="C204" s="23" t="inlineStr">
         <is>
           <t>Anmerkungen</t>
         </is>
       </c>
-      <c r="D150" s="24" t="n"/>
-      <c r="E150" s="24" t="n"/>
-      <c r="F150" s="24" t="n"/>
-      <c r="G150" s="69" t="inlineStr">
+      <c r="D204" s="24" t="n"/>
+      <c r="E204" s="24" t="n"/>
+      <c r="F204" s="24" t="n"/>
+      <c r="G204" s="69" t="inlineStr">
         <is>
           <t>Anmerkungen</t>
         </is>
       </c>
-      <c r="H150" s="24" t="n"/>
-      <c r="I150" s="24" t="n"/>
-      <c r="J150" s="24" t="n"/>
-    </row>
-    <row r="151" hidden="1" outlineLevel="1">
-      <c r="B151" s="35" t="inlineStr">
+      <c r="H204" s="24" t="n"/>
+      <c r="I204" s="24" t="n"/>
+      <c r="J204" s="24" t="n"/>
+    </row>
+    <row r="205">
+      <c r="B205" s="35" t="inlineStr">
         <is>
           <t>Betriebsmittel</t>
         </is>
       </c>
-      <c r="C151" s="36" t="inlineStr">
+      <c r="C205" s="36" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D151" s="37" t="n"/>
-      <c r="E151" s="38" t="n"/>
-      <c r="F151" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G151" s="70" t="inlineStr">
+      <c r="D205" s="37" t="n"/>
+      <c r="E205" s="38" t="n"/>
+      <c r="F205" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G205" s="70" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H151" s="37" t="n"/>
-      <c r="I151" s="38" t="n"/>
-      <c r="J151" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" hidden="1" outlineLevel="1">
-      <c r="B152" s="35" t="inlineStr">
+      <c r="H205" s="37" t="n"/>
+      <c r="I205" s="38" t="n"/>
+      <c r="J205" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="B206" s="35" t="inlineStr">
         <is>
           <t>Werbung / Marketing</t>
         </is>
       </c>
-      <c r="C152" s="25" t="inlineStr">
+      <c r="C206" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D152" s="39" t="n"/>
-      <c r="E152" s="40" t="n"/>
-      <c r="F152" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G152" s="54" t="inlineStr">
+      <c r="D206" s="39" t="n"/>
+      <c r="E206" s="40" t="n"/>
+      <c r="F206" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G206" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H152" s="39" t="n"/>
-      <c r="I152" s="40" t="n"/>
-      <c r="J152" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="153" hidden="1" outlineLevel="1" ht="8.25" customHeight="1">
-      <c r="B153" s="35" t="inlineStr">
+      <c r="H206" s="39" t="n"/>
+      <c r="I206" s="40" t="n"/>
+      <c r="J206" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="B207" s="35" t="inlineStr">
         <is>
           <t>Personalbeschaffung</t>
         </is>
       </c>
-      <c r="C153" s="25" t="inlineStr">
+      <c r="C207" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D153" s="39" t="n"/>
-      <c r="E153" s="40" t="n"/>
-      <c r="F153" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G153" s="54" t="inlineStr">
+      <c r="D207" s="39" t="n"/>
+      <c r="E207" s="40" t="n"/>
+      <c r="F207" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G207" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H153" s="39" t="n"/>
-      <c r="I153" s="40" t="n"/>
-      <c r="J153" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="154" hidden="1" outlineLevel="1" customFormat="1" s="1">
-      <c r="B154" s="35" t="inlineStr">
+      <c r="H207" s="39" t="n"/>
+      <c r="I207" s="40" t="n"/>
+      <c r="J207" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="B208" s="35" t="inlineStr">
         <is>
           <t>Planungskosten</t>
         </is>
       </c>
-      <c r="C154" s="25" t="inlineStr">
+      <c r="C208" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D154" s="39" t="n"/>
-      <c r="E154" s="40" t="n"/>
-      <c r="F154" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G154" s="54" t="inlineStr">
+      <c r="D208" s="39" t="n"/>
+      <c r="E208" s="40" t="n"/>
+      <c r="F208" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G208" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H154" s="39" t="n"/>
-      <c r="I154" s="40" t="n"/>
-      <c r="J154" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="155" hidden="1" outlineLevel="1" ht="6.75" customHeight="1" thickBot="1">
-      <c r="B155" s="35" t="inlineStr">
+      <c r="H208" s="39" t="n"/>
+      <c r="I208" s="40" t="n"/>
+      <c r="J208" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="B209" s="35" t="inlineStr">
         <is>
           <t>Makler</t>
         </is>
       </c>
-      <c r="C155" s="25" t="inlineStr">
+      <c r="C209" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D155" s="39" t="n"/>
-      <c r="E155" s="40" t="n"/>
-      <c r="F155" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G155" s="54" t="inlineStr">
+      <c r="D209" s="39" t="n"/>
+      <c r="E209" s="40" t="n"/>
+      <c r="F209" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G209" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H155" s="39" t="n"/>
-      <c r="I155" s="40" t="n"/>
-      <c r="J155" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156" hidden="1" outlineLevel="1">
-      <c r="B156" s="35" t="inlineStr">
+      <c r="H209" s="39" t="n"/>
+      <c r="I209" s="40" t="n"/>
+      <c r="J209" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="B210" s="35" t="inlineStr">
         <is>
           <t>[Platzhalter]</t>
         </is>
       </c>
-      <c r="C156" s="25" t="inlineStr">
+      <c r="C210" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D156" s="39" t="n"/>
-      <c r="E156" s="40" t="n"/>
-      <c r="F156" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G156" s="54" t="inlineStr">
+      <c r="D210" s="39" t="n"/>
+      <c r="E210" s="40" t="n"/>
+      <c r="F210" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G210" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H156" s="39" t="n"/>
-      <c r="I156" s="40" t="n"/>
-      <c r="J156" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157" collapsed="1">
-      <c r="B157" s="35" t="inlineStr">
+      <c r="H210" s="39" t="n"/>
+      <c r="I210" s="40" t="n"/>
+      <c r="J210" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="B211" s="35" t="inlineStr">
         <is>
           <t>[Platzhalter]</t>
         </is>
       </c>
-      <c r="C157" s="25" t="inlineStr">
+      <c r="C211" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D157" s="39" t="n"/>
-      <c r="E157" s="40" t="n"/>
-      <c r="F157" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G157" s="54" t="inlineStr">
+      <c r="D211" s="39" t="n"/>
+      <c r="E211" s="40" t="n"/>
+      <c r="F211" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G211" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H157" s="39" t="n"/>
-      <c r="I157" s="40" t="n"/>
-      <c r="J157" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="B158" s="35" t="inlineStr">
+      <c r="H211" s="39" t="n"/>
+      <c r="I211" s="40" t="n"/>
+      <c r="J211" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="B212" s="35" t="inlineStr">
         <is>
           <t>[Platzhalter]</t>
         </is>
       </c>
-      <c r="C158" s="25" t="inlineStr">
+      <c r="C212" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D158" s="39" t="n"/>
-      <c r="E158" s="40" t="n"/>
-      <c r="F158" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G158" s="54" t="inlineStr">
+      <c r="D212" s="39" t="n"/>
+      <c r="E212" s="40" t="n"/>
+      <c r="F212" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G212" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H158" s="39" t="n"/>
-      <c r="I158" s="40" t="n"/>
-      <c r="J158" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="B159" s="35" t="inlineStr">
+      <c r="H212" s="39" t="n"/>
+      <c r="I212" s="40" t="n"/>
+      <c r="J212" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="B213" s="35" t="inlineStr">
         <is>
           <t>[Platzhalter]</t>
         </is>
       </c>
-      <c r="C159" s="25" t="inlineStr">
+      <c r="C213" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D159" s="39" t="n"/>
-      <c r="E159" s="40" t="n"/>
-      <c r="F159" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G159" s="54" t="inlineStr">
+      <c r="D213" s="39" t="n"/>
+      <c r="E213" s="40" t="n"/>
+      <c r="F213" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G213" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H159" s="39" t="n"/>
-      <c r="I159" s="40" t="n"/>
-      <c r="J159" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="B160" s="35" t="inlineStr">
+      <c r="H213" s="39" t="n"/>
+      <c r="I213" s="40" t="n"/>
+      <c r="J213" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="B214" s="35" t="inlineStr">
         <is>
           <t>[Platzhalter]</t>
         </is>
       </c>
-      <c r="C160" s="25" t="inlineStr">
+      <c r="C214" s="25" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="D160" s="39" t="n"/>
-      <c r="E160" s="40" t="n"/>
-      <c r="F160" s="50" t="n">
-        <v>0</v>
-      </c>
-      <c r="G160" s="54" t="inlineStr">
+      <c r="D214" s="39" t="n"/>
+      <c r="E214" s="40" t="n"/>
+      <c r="F214" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G214" s="54" t="inlineStr">
         <is>
           <t>XXX</t>
         </is>
       </c>
-      <c r="H160" s="39" t="n"/>
-      <c r="I160" s="40" t="n"/>
-      <c r="J160" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="B161" s="14" t="n"/>
-      <c r="C161" s="15" t="n"/>
-      <c r="D161" s="16" t="n"/>
-      <c r="E161" s="17" t="n"/>
-      <c r="F161" s="17" t="n"/>
-      <c r="G161" s="67" t="n"/>
-      <c r="H161" s="16" t="n"/>
-      <c r="I161" s="17" t="n"/>
-      <c r="J161" s="17" t="n"/>
-    </row>
-    <row r="162">
-      <c r="B162" s="1" t="inlineStr">
+      <c r="H214" s="39" t="n"/>
+      <c r="I214" s="40" t="n"/>
+      <c r="J214" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="B215" s="14" t="n"/>
+      <c r="C215" s="15" t="n"/>
+      <c r="D215" s="16" t="n"/>
+      <c r="E215" s="17" t="n"/>
+      <c r="F215" s="17" t="n"/>
+      <c r="G215" s="67" t="n"/>
+      <c r="H215" s="16" t="n"/>
+      <c r="I215" s="17" t="n"/>
+      <c r="J215" s="17" t="n"/>
+    </row>
+    <row r="216">
+      <c r="B216" s="1" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="C162" s="18" t="n"/>
-      <c r="D162" s="19" t="n"/>
-      <c r="E162" s="20" t="n"/>
-      <c r="F162" s="20">
-        <f>+SUM(F151:F161)</f>
-        <v/>
-      </c>
-      <c r="G162" s="68" t="n"/>
-      <c r="H162" s="19" t="n"/>
-      <c r="I162" s="20" t="n"/>
-      <c r="J162" s="20">
-        <f>+SUM(J151:J161)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="163">
-      <c r="B163" s="7" t="n"/>
-      <c r="C163" s="8" t="n"/>
-      <c r="D163" s="7" t="n"/>
-      <c r="E163" s="7" t="n"/>
-      <c r="F163" s="7" t="n"/>
-      <c r="G163" s="55" t="n"/>
-      <c r="H163" s="7" t="n"/>
-      <c r="I163" s="7" t="n"/>
-      <c r="J163" s="7" t="n"/>
+      <c r="C216" s="18" t="n"/>
+      <c r="D216" s="19" t="n"/>
+      <c r="E216" s="20" t="n"/>
+      <c r="F216" s="20">
+        <f>+SUM(F205:F215)</f>
+        <v/>
+      </c>
+      <c r="G216" s="68" t="n"/>
+      <c r="H216" s="19" t="n"/>
+      <c r="I216" s="20" t="n"/>
+      <c r="J216" s="20">
+        <f>+SUM(J205:J215)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="217">
+      <c r="B217" s="7" t="n"/>
+      <c r="C217" s="8" t="n"/>
+      <c r="D217" s="7" t="n"/>
+      <c r="E217" s="7" t="n"/>
+      <c r="F217" s="7" t="n"/>
+      <c r="G217" s="55" t="n"/>
+      <c r="H217" s="7" t="n"/>
+      <c r="I217" s="7" t="n"/>
+      <c r="J217" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Indexblock: gewichtete Gesamtsteigerung und einheitlicher Mischsatz ergaenzt
Zeile 176 zeigt die gewichtete Steigerung ueber alle acht Positionen
(12,54 Prozent), Zeile 177 den einheitlichen Satz ueber alle Mietflaechen
(14,11 EUR/qm, entspricht 12,87 Prozent gegenueber 12,50 EUR/qm).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Vergleich_Mietkonditionen_JN_DM.xlsx
+++ b/mietkonditionen/Vergleich_Mietkonditionen_JN_DM.xlsx
@@ -553,7 +553,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -944,6 +944,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2007,7 +2010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L217"/>
+  <dimension ref="B2:L217"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col width="3.85546875" customWidth="1" style="2" min="1" max="1"/>
@@ -4956,6 +4959,10 @@
           <t>Summe</t>
         </is>
       </c>
+      <c r="F176" s="136">
+        <f>+IFERROR(I176/H176-1,"")</f>
+        <v/>
+      </c>
       <c r="H176" s="135">
         <f>+SUM(H168:H175)</f>
         <v/>
@@ -4969,7 +4976,17 @@
         <v/>
       </c>
     </row>
-    <row r="177"/>
+    <row r="177">
+      <c r="B177" s="128" t="inlineStr">
+        <is>
+          <t>einheitlicher Satz über alle Mietflächen (€/qm)</t>
+        </is>
+      </c>
+      <c r="C177" s="135">
+        <f>+(I168+I169+I170)/(C168+C169+C170)</f>
+        <v/>
+      </c>
+    </row>
     <row r="178">
       <c r="B178" s="128" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Indexblock auf aktuellen Stand 08/2026 umgestellt
Referenzindex ist der aktuellste amtlich veroeffentlichte Wert: VPI 07/2026
= 125,6 (Destatis, Pressemitteilung PD26_283_611); fuer August 2026 liegt
noch keine Veroeffentlichung vor. Damit liegen alle acht Positionen ueber der
Fuenfprozentschwelle. Gewichtete Steigerung 17,30 Prozent, einheitlicher
Flaechensatz 14,70 EUR/qm gegenueber der Forderung von 14,95 EUR/qm.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Vergleich_Mietkonditionen_JN_DM.xlsx
+++ b/mietkonditionen/Vergleich_Mietkonditionen_JN_DM.xlsx
@@ -4539,7 +4539,7 @@
     <row r="158">
       <c r="B158" s="78" t="inlineStr">
         <is>
-          <t>Berechnung Indexklausel - laut Vermieter beträgt die angepasste Miete 14,95 Euro</t>
+          <t>Berechnung Indexklausel – Stand 08/2026, Referenzindex 07/2026; Forderung Vermieter 14,95 €/qm</t>
         </is>
       </c>
       <c r="G158" s="126" t="n"/>
@@ -4599,11 +4599,11 @@
     <row r="165">
       <c r="B165" s="128" t="inlineStr">
         <is>
-          <t>VPI Referenzmonat (hier 04/2025, frühester Anpassungstermin)</t>
+          <t>VPI Referenzmonat – 07/2026 = 125,6 (aktuellster Stand); 04/2025 = 121,7</t>
         </is>
       </c>
       <c r="C165" s="129" t="n">
-        <v>121.7</v>
+        <v>125.6</v>
       </c>
     </row>
     <row r="166">

</xml_diff>